<commit_message>
Crop Sown Cultivation form: remove the last abbreviation from a validation message
Form version 2026.10.31.1.
</commit_message>
<xml_diff>
--- a/odk/forms/crop_sown_registry_prep.xlsx
+++ b/odk/forms/crop_sown_registry_prep.xlsx
@@ -1416,7 +1416,7 @@
       </c>
       <c r="G30" s="39" t="inlineStr">
         <is>
-          <t>Actual Cultivated Date (GC) must be between Start Date and End Date.</t>
+          <t>Actual Cultivated Date must be between Start Date and End Date.</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="C2" s="39" t="inlineStr">
         <is>
-          <t>2026.10.31</t>
+          <t>2026.10.31.1</t>
         </is>
       </c>
       <c r="D2" s="39" t="inlineStr">

</xml_diff>

<commit_message>
Crop Sown Cultivation form: remove the last abbreviation from a validation message (#183)
Form version 2026.10.31.1.
</commit_message>
<xml_diff>
--- a/odk/forms/crop_sown_registry_prep.xlsx
+++ b/odk/forms/crop_sown_registry_prep.xlsx
@@ -1416,7 +1416,7 @@
       </c>
       <c r="G30" s="39" t="inlineStr">
         <is>
-          <t>Actual Cultivated Date (GC) must be between Start Date and End Date.</t>
+          <t>Actual Cultivated Date must be between Start Date and End Date.</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="C2" s="39" t="inlineStr">
         <is>
-          <t>2026.10.31</t>
+          <t>2026.10.31.1</t>
         </is>
       </c>
       <c r="D2" s="39" t="inlineStr">

</xml_diff>